<commit_message>
Unlock paid Excel workbooks so buyers can edit them.
Sheet and workbook protection blocked data entry. Files are the same
templates with protection removed.
</commit_message>
<xml_diff>
--- a/content/spreadsheets/Online-Seller-Profit-Tracker.xlsx
+++ b/content/spreadsheets/Online-Seller-Profit-Tracker.xlsx
@@ -2,7 +2,6 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -3265,7 +3264,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="85">
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="G21:H21"/>
@@ -11609,7 +11607,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <autoFilter ref="A4:N204"/>
   <mergeCells count="4">
     <mergeCell ref="A1:P1"/>
@@ -12773,7 +12770,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <autoFilter ref="A4:J34"/>
   <mergeCells count="5">
     <mergeCell ref="A1:J1"/>
@@ -14074,7 +14070,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <autoFilter ref="A4:F84"/>
   <mergeCells count="4">
     <mergeCell ref="A3:G3"/>
@@ -16466,7 +16461,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <autoFilter ref="A4:K52"/>
   <mergeCells count="3">
     <mergeCell ref="A2:K2"/>
@@ -17584,7 +17578,6 @@
       <c r="H90" s="9" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="42">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B14:G14"/>

</xml_diff>